<commit_message>
Planilha: links do Instagram via Stract
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GQAEiUYJHrFswFx8FRgado
</commit_message>
<xml_diff>
--- a/top_anuncios_contrate_um_subido.xlsx
+++ b/top_anuncios_contrate_um_subido.xlsx
@@ -448,8 +448,8 @@
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="70" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -496,12 +496,12 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>ID da mídia no Instagram</t>
+          <t>ID do anúncio do link</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Link do anúncio (Gerenciador)</t>
+          <t>Link do Instagram</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -541,14 +541,10 @@
       <c r="H2" s="3" t="n">
         <v>0.9291338582677166</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>18031752928618872</t>
-        </is>
-      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6304454990162</t>
+          <t>não disponível (anúncio deletado)</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -588,14 +584,10 @@
       <c r="H3" s="3" t="n">
         <v>0.3398826231181424</v>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>18031752928618872</t>
-        </is>
-      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6304454990162</t>
+          <t>não disponível (anúncio deletado)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -637,12 +629,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>17843337936262504</t>
+          <t>6535156139562</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6535156139562</t>
+          <t>https://www.instagram.com/p/C9dlrMINu4q/</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -684,12 +676,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>18055040860485962</t>
+          <t>6535156126562</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6535156126562</t>
+          <t>https://www.instagram.com/p/CzCMnz6t_tb/</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -731,12 +723,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>18296061268164432</t>
+          <t>6535156139962</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6535156139962</t>
+          <t>https://www.instagram.com/p/C9dlpeHNYml/</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -778,12 +770,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>18049101511464180</t>
+          <t>6535154856362</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6461506853762</t>
+          <t>https://www.instagram.com/p/C9i22vut3my/  (de outro anúncio da mesma criativa; o original foi deletado)</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -825,12 +817,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>18296061268164432</t>
+          <t>6535156139962</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6535156139962</t>
+          <t>https://www.instagram.com/p/C9dlpeHNYml/</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -872,12 +864,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>18055040860485962</t>
+          <t>6535156126562</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6535156126562</t>
+          <t>https://www.instagram.com/p/CzCMnz6t_tb/</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -919,12 +911,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>17843337936262504</t>
+          <t>6535156139562</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6535156139562</t>
+          <t>https://www.instagram.com/p/C9dlrMINu4q/</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -966,12 +958,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>17974103582440074</t>
+          <t>6535156136762</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6535156136762</t>
+          <t>https://www.instagram.com/p/CzCctZUNr3A/</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1013,12 +1005,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>18023349754773982</t>
+          <t>6535156137162</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6535156137162</t>
+          <t>https://www.instagram.com/p/CzCcUf6NloD/</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1060,12 +1052,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>18028401347213789</t>
+          <t>6578629449562</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6578629449562</t>
+          <t>https://www.instagram.com/p/C-T0lblN0hI/</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1107,12 +1099,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>18072878170594122</t>
+          <t>6535156128362</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6535156128362</t>
+          <t>https://www.instagram.com/p/DBKPYigMP7r/</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1154,12 +1146,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>18055040860485962</t>
+          <t>6535156126562</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6535156126562</t>
+          <t>https://www.instagram.com/p/CzCMnz6t_tb/</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1201,12 +1193,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>18028627813658773</t>
+          <t>6535156136562</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6535156136562</t>
+          <t>https://www.instagram.com/p/CzCdcJQNgGZ/</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1248,12 +1240,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>17974103582440074</t>
+          <t>6535156136762</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6535156136762</t>
+          <t>https://www.instagram.com/p/CzCctZUNr3A/</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1295,12 +1287,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>18191417041324808</t>
+          <t>6646114026162</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6646114026162</t>
+          <t>https://www.instagram.com/p/DF--tWTMTqr/</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1342,12 +1334,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>17950379879895192</t>
+          <t>6592749588962</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6592749588962</t>
+          <t>https://www.instagram.com/p/DDaf_MRsk4a/</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1389,12 +1381,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>17853292626387926</t>
+          <t>6646114024562</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6646114024562</t>
+          <t>https://www.instagram.com/p/DF--sk-MdJ8/</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1436,12 +1428,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>18258491662282311</t>
+          <t>6592730909962</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6592730909962</t>
+          <t>https://www.instagram.com/p/DDaf2-oMnA1/</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1483,12 +1475,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>17888222445083169</t>
+          <t>6592732576762</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=498598010251531&amp;selected_ad_ids=6592732576762</t>
+          <t>https://www.instagram.com/p/DDaf4MTs_Ti/</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1530,12 +1522,12 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>17877323400369419</t>
+          <t>120227522250920656</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=328928844722088&amp;selected_ad_ids=120227522250920656</t>
+          <t>https://www.instagram.com/p/DMsYPb7Aq6-/</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1577,12 +1569,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>18287179297281279</t>
+          <t>120229757620750656</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=328928844722088&amp;selected_ad_ids=120229757620750656</t>
+          <t>https://www.instagram.com/p/DOdrNY0ADDQ/</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -1624,12 +1616,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>18062105948193925</t>
+          <t>120227522250890656</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=328928844722088&amp;selected_ad_ids=120227522250890656</t>
+          <t>https://www.instagram.com/p/DMsYPlUgsH4/</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -1671,12 +1663,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>17967723848952539</t>
+          <t>120229758057570656</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=328928844722088&amp;selected_ad_ids=120229758057570656</t>
+          <t>https://www.instagram.com/p/DOdrvusgJZR/</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -1718,12 +1710,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>17979787742763830</t>
+          <t>120231241992690656</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=328928844722088&amp;selected_ad_ids=120231241992690656</t>
+          <t>https://www.instagram.com/p/DPnL9BJgCXK/</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -1765,12 +1757,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>18287179297281279</t>
+          <t>120229757620750656</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=328928844722088&amp;selected_ad_ids=120229757620750656</t>
+          <t>https://www.instagram.com/p/DOdrNY0ADDQ/</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -1812,12 +1804,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>17913093807273581</t>
+          <t>120236424751510656</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=328928844722088&amp;selected_ad_ids=120236424751510656</t>
+          <t>https://www.instagram.com/p/DTlGt9NAO1R/</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -1859,12 +1851,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>18062105948193925</t>
+          <t>120227522250890656</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=328928844722088&amp;selected_ad_ids=120227522250890656</t>
+          <t>https://www.instagram.com/p/DMsYPlUgsH4/</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -1906,12 +1898,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>18082353800232327</t>
+          <t>120236424751500656</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=328928844722088&amp;selected_ad_ids=120236424751500656</t>
+          <t>https://www.instagram.com/p/DTlGumTAPJe/</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -1953,12 +1945,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>17979787742763830</t>
+          <t>120231241992690656</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=328928844722088&amp;selected_ad_ids=120231241992690656</t>
+          <t>https://www.instagram.com/p/DPnL9BJgCXK/</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2000,12 +1992,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>18625185046061472</t>
+          <t>120247489968710656</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/adsmanager/manage/ads/edit?act=328928844722088&amp;selected_ad_ids=120247489968710656</t>
+          <t>https://www.instagram.com/p/DcxYJkpASQt/</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2359,7 +2351,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Link do Instagram: o conector não expõe o permalink (instagram.com/p/...) dos posts usados nos anúncios; foi possível obter apenas o ID da mídia (effective_instagram_media_id) e o link do anúncio no Gerenciador.</t>
+          <t>Link do Instagram: permalink do post gerado pelo anúncio (extração do Stract, campo creative.instagram_permalink_url), usando o ID de anúncio de maior investimento de cada criativo. Cada anúncio/conjunto gera um post diferente, então outros IDs do mesmo criativo têm outros links.</t>
         </is>
       </c>
     </row>

</xml_diff>